<commit_message>
Add Robus Predictor benchmark script and documentation files
</commit_message>
<xml_diff>
--- a/Documentacion/Carta Gantt RobusPredictor.xlsx
+++ b/Documentacion/Carta Gantt RobusPredictor.xlsx
@@ -183,7 +183,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -200,6 +200,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF93C47D"/>
         <bgColor rgb="FF93C47D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAD3"/>
+        <bgColor rgb="FFD9EAD3"/>
       </patternFill>
     </fill>
     <fill>
@@ -422,15 +428,15 @@
     <xf borderId="4" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="5" fillId="4" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="6" fillId="4" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="4" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="5" fillId="5" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="6" fillId="5" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="6" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="6" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
@@ -447,21 +453,21 @@
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="5" fillId="5" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="6" fillId="5" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="5" fillId="6" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="6" fillId="6" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="6" fillId="6" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="6" fillId="7" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="6" fillId="8" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="6" fillId="8" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="6" fillId="9" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -470,23 +476,23 @@
     </xf>
     <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="6" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="6" fillId="8" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="6" fillId="9" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="6" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="6" fillId="7" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="7" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="7" fillId="7" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -504,10 +510,10 @@
     <xf borderId="9" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="9" fillId="9" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="9" fillId="10" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="10" fillId="9" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="10" fillId="10" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -724,7 +730,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8.13"/>
-    <col customWidth="1" min="2" max="2" width="40.38"/>
+    <col customWidth="1" min="2" max="2" width="46.25"/>
     <col customWidth="1" min="3" max="26" width="10.63"/>
   </cols>
   <sheetData>

</xml_diff>